<commit_message>
feat(pricing): WhatsApp con cargos de Meta incluidos + paquete de difusión
- Plan incluye conversaciones, recordatorios y 500 mensajes de difusión al mes;
  OrzaTech absorbe los cargos de Meta (método de pago de OrzaTech en la WABA)
- Nuevo extra: paquete de 1,000 mensajes de difusión por $1,200, en la misma factura
- Precios (FAQ), playbook (objeción nueva), README de ventas, cotizador y
  checklist de entrega actualizados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sales/cotizador.xlsx
+++ b/sales/cotizador.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Precios" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Propuesta'!$A$1:$D$41</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Propuesta'!$A$1:$D$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -519,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -629,313 +629,334 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Forma de pago de la mensualidad</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Mensual</t>
-        </is>
+          <t>Paquetes de difusión WhatsApp (1,000 msj)</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Escalón de implementación</t>
+          <t>Forma de pago de la mensualidad</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>A · Lista</t>
+          <t>Mensual</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Vendedor</t>
+          <t>Escalón de implementación</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Nombre del vendedor</t>
+          <t>A · Lista</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
+          <t>Vendedor</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Nombre del vendedor</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
           <t>Fecha de la propuesta</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Ejemplo precargado: sobrescribe con los datos reales.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>RECOMENDACIÓN DE HORAS</t>
         </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Minutos estimados al mes</t>
-        </is>
-      </c>
-      <c r="B19" s="7">
-        <f>$B$9*Precios!$B$10</f>
-        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
+          <t>Minutos estimados al mes</t>
+        </is>
+      </c>
+      <c r="B20" s="7">
+        <f>$B$9*Precios!$B$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
           <t>Horas estimadas al mes</t>
         </is>
       </c>
-      <c r="B20" s="8">
-        <f>$B$19/60</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="B21" s="8">
+        <f>$B$20/60</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>Paquete recomendado</t>
         </is>
       </c>
-      <c r="B21" s="10">
-        <f>IF($B$20&lt;=5,"Ninguno",IF($B$20&lt;=10,"+5 h","+10 h"))</f>
-        <v/>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="B22" s="10">
+        <f>IF($B$21&lt;=5,"Ninguno",IF($B$21&lt;=10,"+5 h","+10 h"))</f>
+        <v/>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>5 h incluidas; arriba de 15 h estimadas, platícalo con tu líder</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>MENSUALIDAD</t>
         </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Plan Innmobi</t>
-        </is>
-      </c>
-      <c r="B24" s="11">
-        <f>Precios!$B$4</f>
-        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Paquete de voz</t>
+          <t>Plan Innmobi</t>
         </is>
       </c>
       <c r="B25" s="11">
-        <f>INDEX(Precios!$C$15:$C$17,MATCH($B$10,Precios!$A$15:$A$17,0))</f>
+        <f>Precios!$B$4</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
+          <t>Paquete de voz</t>
+        </is>
+      </c>
+      <c r="B26" s="11">
+        <f>INDEX(Precios!$C$15:$C$17,MATCH($B$10,Precios!$A$15:$A$17,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
           <t>Líneas adicionales</t>
         </is>
       </c>
-      <c r="B26" s="11">
+      <c r="B27" s="11">
         <f>$B$11*Precios!$B$8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>Subtotal mensual</t>
-        </is>
-      </c>
-      <c r="B27" s="12">
-        <f>$B$24+$B$25+$B$26</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>IVA</t>
+          <t>Paquetes de difusión WhatsApp</t>
         </is>
       </c>
       <c r="B28" s="11">
-        <f>$B$27*Precios!$B$7</f>
+        <f>$B$12*Precios!$B$9</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>Total mensual con IVA</t>
-        </is>
-      </c>
-      <c r="B29" s="13">
-        <f>$B$27+$B$28</f>
+          <t>Subtotal mensual</t>
+        </is>
+      </c>
+      <c r="B29" s="12">
+        <f>$B$25+$B$26+$B$27+$B$28</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
+          <t>IVA</t>
+        </is>
+      </c>
+      <c r="B30" s="11">
+        <f>$B$29*Precios!$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>Total mensual con IVA</t>
+        </is>
+      </c>
+      <c r="B31" s="13">
+        <f>$B$29+$B$30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
           <t>Si paga anual: total del año sin IVA</t>
         </is>
       </c>
-      <c r="B30" s="11">
-        <f>$B$24*Precios!$B$5+($B$25+$B$26)*12</f>
-        <v/>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="B32" s="11">
+        <f>$B$25*Precios!$B$5+($B$26+$B$27+$B$28)*12</f>
+        <v/>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Plan: 12 meses por el precio de 10; extras completos</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Si paga anual: total del año con IVA</t>
         </is>
       </c>
-      <c r="B31" s="11">
-        <f>$B$30*(1+Precios!$B$7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="B33" s="11">
+        <f>$B$32*(1+Precios!$B$7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>IMPLEMENTACIÓN</t>
         </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>Al firmar</t>
-        </is>
-      </c>
-      <c r="B34" s="11">
-        <f>INDEX(Precios!$B$22:$B$25,MATCH($B$13,Precios!$A$22:$A$25,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>Segundo pago</t>
-        </is>
-      </c>
-      <c r="B35" s="11">
-        <f>INDEX(Precios!$C$22:$C$25,MATCH($B$13,Precios!$A$22:$A$25,0))</f>
-        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Cuándo se paga el segundo pago</t>
-        </is>
-      </c>
-      <c r="B36" s="14">
-        <f>INDEX(Precios!$D$22:$D$25,MATCH($B$13,Precios!$A$22:$A$25,0))</f>
+          <t>Al firmar</t>
+        </is>
+      </c>
+      <c r="B36" s="11">
+        <f>INDEX(Precios!$B$22:$B$25,MATCH($B$14,Precios!$A$22:$A$25,0))</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Condición del escalón</t>
-        </is>
-      </c>
-      <c r="B37" s="14">
-        <f>INDEX(Precios!$E$22:$E$25,MATCH($B$13,Precios!$A$22:$A$25,0))</f>
+          <t>Segundo pago</t>
+        </is>
+      </c>
+      <c r="B37" s="11">
+        <f>INDEX(Precios!$C$22:$C$25,MATCH($B$14,Precios!$A$22:$A$25,0))</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
+          <t>Cuándo se paga el segundo pago</t>
+        </is>
+      </c>
+      <c r="B38" s="14">
+        <f>INDEX(Precios!$D$22:$D$25,MATCH($B$14,Precios!$A$22:$A$25,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Condición del escalón</t>
+        </is>
+      </c>
+      <c r="B39" s="14">
+        <f>INDEX(Precios!$E$22:$E$25,MATCH($B$14,Precios!$A$22:$A$25,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
           <t>Revisión (debe sumar la implementación)</t>
         </is>
       </c>
-      <c r="B38" s="14">
-        <f>IF($B$34+$B$35=Precios!$B$6,"OK","REVISAR")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
+      <c r="B40" s="14">
+        <f>IF($B$36+$B$37=Precios!$B$6,"OK","REVISAR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
         <is>
           <t>PAGOS</t>
         </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="9" t="inlineStr">
-        <is>
-          <t>Primer pago (al firmar) sin IVA</t>
-        </is>
-      </c>
-      <c r="B41" s="12">
-        <f>$B$34+IF($B$12="Anual",$B$30,$B$27)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="9" t="inlineStr">
-        <is>
-          <t>Primer pago con IVA</t>
-        </is>
-      </c>
-      <c r="B42" s="13">
-        <f>$B$41*(1+Precios!$B$7)</f>
-        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>Total primer año sin IVA</t>
+          <t>Primer pago (al firmar) sin IVA</t>
         </is>
       </c>
       <c r="B43" s="12">
-        <f>Precios!$B$6+IF($B$12="Anual",$B$30,$B$27*12)</f>
+        <f>$B$36+IF($B$13="Anual",$B$32,$B$29)</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>Total primer año con IVA</t>
+          <t>Primer pago con IVA</t>
         </is>
       </c>
       <c r="B44" s="13">
         <f>$B$43*(1+Precios!$B$7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>Total primer año sin IVA</t>
+        </is>
+      </c>
+      <c r="B45" s="12">
+        <f>Precios!$B$6+IF($B$13="Anual",$B$32,$B$29*12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>Total primer año con IVA</t>
+        </is>
+      </c>
+      <c r="B46" s="13">
+        <f>$B$45*(1+Precios!$B$7)</f>
         <v/>
       </c>
     </row>
@@ -944,13 +965,13 @@
     <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>=Precios!$A$15:$A$17</formula1>
     </dataValidation>
-    <dataValidation sqref="B12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Mensual,Anual"</formula1>
     </dataValidation>
-    <dataValidation sqref="B13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>=Precios!$A$22:$A$25</formula1>
     </dataValidation>
-    <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="whole" operator="between">
+    <dataValidation sqref="B11 B12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>20</formula2>
     </dataValidation>
@@ -965,7 +986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:D41"/>
+  <dimension ref="B2:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -996,7 +1017,7 @@
     </row>
     <row r="6">
       <c r="B6" s="2">
-        <f>Cotizador!$B$7&amp;" · "&amp;Cotizador!$B$8&amp;" asesores · Fecha: "&amp;Cotizador!$B$15&amp;" · Vigencia: "&amp;Precios!$B$11&amp;" días"</f>
+        <f>Cotizador!$B$7&amp;" · "&amp;Cotizador!$B$8&amp;" asesores · Fecha: "&amp;Cotizador!$B$16&amp;" · Vigencia: "&amp;Precios!$B$12&amp;" días"</f>
         <v/>
       </c>
     </row>
@@ -1052,46 +1073,39 @@
     <row r="15">
       <c r="B15" s="4" t="inlineStr">
         <is>
+          <t>✓  WhatsApp con los cargos de Meta incluidos y 500 mensajes de difusión al mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="4" t="inlineStr">
+        <is>
           <t>✓  Soporte directo vía WhatsApp con el equipo que construye el producto</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="3" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Inversión mensual</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>MXN sin IVA</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>MXN con IVA</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="17" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Plan Innmobi</t>
         </is>
-      </c>
-      <c r="C18" s="18">
-        <f>Cotizador!$B$24</f>
-        <v/>
-      </c>
-      <c r="D18" s="18">
-        <f>Cotizador!$B$24*(1+Precios!$B$7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="17">
-        <f>"Paquete de voz: "&amp;Cotizador!$B$10</f>
-        <v/>
       </c>
       <c r="C19" s="18">
         <f>Cotizador!$B$25</f>
@@ -1104,7 +1118,7 @@
     </row>
     <row r="20">
       <c r="B20" s="17">
-        <f>"Líneas adicionales: "&amp;Cotizador!$B$11</f>
+        <f>"Paquete de voz: "&amp;Cotizador!$B$10</f>
         <v/>
       </c>
       <c r="C20" s="18">
@@ -1117,165 +1131,193 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="19" t="inlineStr">
+      <c r="B21" s="17">
+        <f>"Líneas adicionales: "&amp;Cotizador!$B$11</f>
+        <v/>
+      </c>
+      <c r="C21" s="18">
+        <f>Cotizador!$B$27</f>
+        <v/>
+      </c>
+      <c r="D21" s="18">
+        <f>Cotizador!$B$27*(1+Precios!$B$7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="17">
+        <f>"Difusión WhatsApp extra: "&amp;Cotizador!$B$12&amp;" x 1,000 mensajes"</f>
+        <v/>
+      </c>
+      <c r="C22" s="18">
+        <f>Cotizador!$B$28</f>
+        <v/>
+      </c>
+      <c r="D22" s="18">
+        <f>Cotizador!$B$28*(1+Precios!$B$7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="19" t="inlineStr">
         <is>
           <t>Total mensual</t>
         </is>
       </c>
-      <c r="C21" s="20">
-        <f>Cotizador!$B$27</f>
-        <v/>
-      </c>
-      <c r="D21" s="20">
-        <f>Cotizador!$B$27*(1+Precios!$B$7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="2">
-        <f>IF(Cotizador!$B$12="Anual","Pago anual elegido: "&amp;TEXT(Cotizador!$B$30,"$#,##0")&amp;" + IVA por 12 meses (12 por el precio de 10 en el plan)","Opción anual: 12 meses por el precio de 10 en el plan")</f>
+      <c r="C23" s="20">
+        <f>Cotizador!$B$29</f>
+        <v/>
+      </c>
+      <c r="D23" s="20">
+        <f>Cotizador!$B$29*(1+Precios!$B$7)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="2">
+        <f>IF(Cotizador!$B$13="Anual","Pago anual elegido: "&amp;TEXT(Cotizador!$B$32,"$#,##0")&amp;" + IVA por 12 meses (12 por el precio de 10 en el plan)","Opción anual: 12 meses por el precio de 10 en el plan")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Implementación (pago único)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="21" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="21" t="inlineStr">
         <is>
           <t>Implementación: migración, canales y onboarding 4 semanas</t>
         </is>
       </c>
-      <c r="C25" s="22">
+      <c r="C27" s="22">
         <f>Precios!$B$6</f>
         <v/>
       </c>
-      <c r="D25" s="22">
+      <c r="D27" s="22">
         <f>Precios!$B$6*(1+Precios!$B$7)</f>
         <v/>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="17" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>Al firmar</t>
         </is>
       </c>
-      <c r="C26" s="23">
-        <f>Cotizador!$B$34</f>
-        <v/>
-      </c>
-      <c r="D26" s="23">
-        <f>Cotizador!$B$34*(1+Precios!$B$7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="17">
-        <f>IF(Cotizador!$B$35=0,"Sin segundo pago","Segundo pago: "&amp;Cotizador!$B$36)</f>
-        <v/>
-      </c>
-      <c r="C27" s="23">
-        <f>Cotizador!$B$35</f>
-        <v/>
-      </c>
-      <c r="D27" s="23">
-        <f>Cotizador!$B$35*(1+Precios!$B$7)</f>
+      <c r="C28" s="23">
+        <f>Cotizador!$B$36</f>
+        <v/>
+      </c>
+      <c r="D28" s="23">
+        <f>Cotizador!$B$36*(1+Precios!$B$7)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" s="17">
+        <f>IF(Cotizador!$B$37=0,"Sin segundo pago","Segundo pago: "&amp;Cotizador!$B$38)</f>
+        <v/>
+      </c>
+      <c r="C29" s="23">
+        <f>Cotizador!$B$37</f>
+        <v/>
+      </c>
+      <c r="D29" s="23">
+        <f>Cotizador!$B$37*(1+Precios!$B$7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Resumen de pagos</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="19" t="inlineStr">
+    <row r="32">
+      <c r="B32" s="19" t="inlineStr">
         <is>
           <t>Primer pago (al firmar)</t>
         </is>
       </c>
-      <c r="C30" s="20">
-        <f>Cotizador!$B$41</f>
-        <v/>
-      </c>
-      <c r="D30" s="20">
-        <f>Cotizador!$B$41*(1+Precios!$B$7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="21" t="inlineStr">
+      <c r="C32" s="20">
+        <f>Cotizador!$B$43</f>
+        <v/>
+      </c>
+      <c r="D32" s="20">
+        <f>Cotizador!$B$43*(1+Precios!$B$7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="21" t="inlineStr">
         <is>
           <t>Total del primer año</t>
         </is>
       </c>
-      <c r="C31" s="22">
-        <f>Cotizador!$B$43</f>
-        <v/>
-      </c>
-      <c r="D31" s="22">
-        <f>Cotizador!$B$43*(1+Precios!$B$7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="3" t="inlineStr">
+      <c r="C33" s="22">
+        <f>Cotizador!$B$45</f>
+        <v/>
+      </c>
+      <c r="D33" s="22">
+        <f>Cotizador!$B$45*(1+Precios!$B$7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Condiciones</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="24" t="inlineStr">
-        <is>
-          <t>·  Precios en pesos mexicanos más IVA. Facturamos con CFDI desde OrzaTech S.A.P.I. de C.V.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="24" t="inlineStr">
-        <is>
-          <t>·  La implementación arranca con el pago de firma. Duración: 4 semanas.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="24" t="inlineStr">
         <is>
-          <t>·  Horas de llamadas no usadas no se acumulan. Minuto adicional sin paquete: $6 MXN + IVA.</t>
+          <t>·  Precios en pesos mexicanos más IVA. Facturamos con CFDI desde OrzaTech S.A.P.I. de C.V.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="24" t="inlineStr">
         <is>
-          <t>·  Los cargos de Meta por mensajes de WhatsApp se cobran directo a la cuenta de Meta de la inmobiliaria.</t>
+          <t>·  La implementación arranca con el pago de firma. Duración: 4 semanas.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="24" t="inlineStr">
         <is>
+          <t>·  Horas de llamadas no usadas no se acumulan. Minuto adicional sin paquete: $6 MXN + IVA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="24" t="inlineStr">
+        <is>
+          <t>·  Los cargos de Meta por WhatsApp están incluidos (conversaciones, recordatorios y 500 mensajes de difusión al mes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="24" t="inlineStr">
+        <is>
           <t>·  Sin lock-in: si te vas, exportamos tu data en CSV/JSON y la borramos de nuestros servidores en 30 días.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="B39" s="2">
-        <f>IF(Cotizador!$B$35=0,"","·  Condición del calendario de pago elegido: "&amp;Cotizador!$B$37&amp;".")</f>
-        <v/>
-      </c>
-    </row>
     <row r="41">
-      <c r="B41" s="9">
-        <f>"Tu contacto: "&amp;Cotizador!$B$14&amp;" · ventas@innmobi.ai · WhatsApp +52 56 2059 5320"</f>
+      <c r="B41" s="2">
+        <f>IF(Cotizador!$B$37=0,"","·  Condición del calendario de pago elegido: "&amp;Cotizador!$B$39&amp;".")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="9">
+        <f>"Tu contacto: "&amp;Cotizador!$B$15&amp;" · ventas@innmobi.ai · WhatsApp +52 56 2059 5320"</f>
         <v/>
       </c>
     </row>
@@ -1395,43 +1437,58 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Minuto de voz sin paquete</t>
+          <t>Paquete de 1,000 mensajes de difusión WhatsApp</t>
         </is>
       </c>
       <c r="B9" s="26" t="n">
-        <v>6</v>
+        <v>1200</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Se cobra al cierre de mes si se pasan de sus horas</t>
+          <t>Incluidos 500 al mes; este paquete agrega 1,000</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Minutos por llamada de calificación (promedio)</t>
-        </is>
-      </c>
-      <c r="B10" s="29" t="n">
-        <v>2.5</v>
+          <t>Minuto de voz sin paquete</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="n">
+        <v>6</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Para estimar horas</t>
+          <t>Se cobra al cierre de mes si se pasan de sus horas</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
+          <t>Minutos por llamada de calificación (promedio)</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Para estimar horas</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
           <t>Vigencia de la propuesta (días)</t>
         </is>
       </c>
-      <c r="B11" s="27" t="n">
+      <c r="B12" s="27" t="n">
         <v>14</v>
       </c>
-      <c r="C11" s="2" t="inlineStr"/>
+      <c r="C12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">

</xml_diff>